<commit_message>
This is my 2nd commit
</commit_message>
<xml_diff>
--- a/target/test-classes/TestData/ExcelData.xlsx
+++ b/target/test-classes/TestData/ExcelData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kburada\eclipse-workspace\ert\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F483A1C7-FCC5-435C-956C-8DAB1248933E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D09D02B-E46B-4CB4-9ABD-AE082E69B481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{40BD7AF7-E067-4703-BE56-9A67774EBF2A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>UserName</t>
   </si>
@@ -64,6 +64,21 @@
   </si>
   <si>
     <t>Budugu</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Name2</t>
+  </si>
+  <si>
+    <t>Name3</t>
+  </si>
+  <si>
+    <t>Name4</t>
+  </si>
+  <si>
+    <t>Test1</t>
   </si>
 </sst>
 </file>
@@ -448,29 +463,44 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD739C9D-47E9-4168-A407-C7FF6D2F06B2}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
       <c r="B1" t="s">
         <v>5</v>
       </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2">
         <v>400</v>
       </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -478,7 +508,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>

</xml_diff>